<commit_message>
Revise SysRS wording, add notes to diagrams and test cases, expand README
</commit_message>
<xml_diff>
--- a/04-Decision-Matrix/SHSS_Decision_Matrices.xlsx
+++ b/04-Decision-Matrix/SHSS_Decision_Matrices.xlsx
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="20" min="1" max="1"/>
@@ -740,113 +740,125 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="23" t="inlineStr"/>
-      <c r="B6" s="22" t="inlineStr"/>
+    <row r="6" ht="60" customHeight="1" s="20">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>How I scored</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>The scores are my own judgement from data sheets, product reviews and, for a few of the devices, hands-on use. I filled in the weights first and the scores afterwards so that the weighting could not be tuned towards a favourite option. Where two options were close I say so in the final-decision text instead of pretending the numbers settle it.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr"/>
+      <c r="B7" s="22" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Matrix (tab)</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Selected alternative (Total Score)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="23" t="inlineStr">
-        <is>
-          <t>Motion Sensors</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="inlineStr">
-        <is>
-          <t>PIR motion sensor, Zigbee 3.0, pet-immune (4.40)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>Door-Window Sensors</t>
+          <t>Motion Sensors</t>
         </is>
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Magnetic reed contact sensor, Zigbee 3.0 (4.65)</t>
+          <t>PIR motion sensor, Zigbee 3.0, pet-immune (4.40)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>Water Leak Sensors</t>
+          <t>Door-Window Sensors</t>
         </is>
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>Zigbee spot leak sensor with probe cable (4.75)</t>
+          <t>Magnetic reed contact sensor, Zigbee 3.0 (4.65)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>Cameras</t>
+          <t>Water Leak Sensors</t>
         </is>
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>PoE wired IP camera (ONVIF/RTSP) (4.30)</t>
+          <t>Zigbee spot leak sensor with probe cable (4.75)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>Controllers - Smart Lock</t>
+          <t>Cameras</t>
         </is>
       </c>
       <c r="B12" s="22" t="inlineStr">
         <is>
-          <t>Zigbee smart lock (4.35)</t>
+          <t>PoE wired IP camera (ONVIF/RTSP) (4.30)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>Controllers - Lighting</t>
+          <t>Controllers - Smart Lock</t>
         </is>
       </c>
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t>Zigbee smart bulb / switch (4.85)</t>
+          <t>Zigbee smart lock (4.35)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>Controllers - Siren</t>
+          <t>Controllers - Lighting</t>
         </is>
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>Wired 12 V siren on CCU relay output (4.20)</t>
+          <t>Zigbee smart bulb / switch (4.85)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
+          <t>Controllers - Siren</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Wired 12 V siren on CCU relay output (4.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
           <t>Server - Local vs Cloud</t>
         </is>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Hybrid: local-first server + cloud relay (remote access, push, backup) (3.95)</t>
         </is>
@@ -1247,7 +1259,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 1 – PIR motion sensor, Zigbee 3.0, pet-immune. It scores highest overall because it combines good detection accuracy with pet/HVAC false-alarm immunity (the two heaviest criteria), multi-year battery life on a coin cell and the lowest unit cost, while joining the Zigbee hub natively without an extra radio. The dual-technology Z-Wave sensor detects slightly better but needs a second Z-Wave controller, costs about twice as much and drains batteries faster. The Wi-Fi microwave sensor is mains-dependent, prone to false alarms through walls and adds load to the home Wi-Fi.</t>
+          <t>I picked Option 1, the pet-immune PIR on Zigbee 3.0. It is not the most sensitive of the three, but detection accuracy and false-alarm immunity are the two criteria I weighted most, and the PIR is the only option that is good at both without a compromise elsewhere: a coin cell lasts two to three years and it joins the hub's Zigbee mesh directly. The dual-technology PIR+microwave sensor is technically the best detector, but it is Z-Wave, so it would need a second radio in the CCU, costs about twice as much and eats batteries. The Wi-Fi microwave sensor I scored low on purpose: it needs mains power, it sees through thin walls (false alarms from the neighbour's corridor) and it adds yet another device to the home Wi-Fi.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -2667,7 +2679,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 1 – Magnetic reed contact sensor, Zigbee 3.0. It leads on the heaviest-weighted criteria – installation ease (peel-and-stick, no wiring), reliability and protocol fit with the Zigbee hub – and offers multi-year battery life at the lowest unit cost. The wired contact is the most reliable and best supervised option, but running cable to every door and window is impractical in a retrofit home. The Wi-Fi sensor drains its battery in months and bypasses the hub's local mesh.</t>
+          <t>Option 1, the Zigbee reed contact, is the clear winner and honestly the obvious choice for a retrofit home: peel-and-stick installation, two to three years on a battery, cheap enough to put on every window, and native to the hub. I gave the wired contact top marks for reliability and supervision, and if this were a new build with cable already in the walls I would choose it. The Wi-Fi contact sensor loses on battery life (months, not years) and because it talks to the vendor cloud instead of the local mesh.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -4087,7 +4099,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 1 – Zigbee spot leak sensor with probe cable. It wins on battery life (years on a coin cell), protocol fit with the hub, unit cost and placement flexibility: the probe cable reaches under appliances and into tight spaces where a wired or bulky Wi-Fi unit cannot go. The wired probe is reliable but requires cable runs to the CCU panel from every wet location. The Wi-Fi sensor needs frequent recharging and depends on Wi-Fi coverage in basements and utility rooms.</t>
+          <t>Option 1 again: the Zigbee spot sensor with a probe cable. What decided it for me was placement. Leaks happen under the dishwasher, behind the washing machine and under the water heater, and the probe cable reaches places where a boxy Wi-Fi unit does not fit. Battery life and cost are in the same league as the other Zigbee sensors. The wired probe is reliable but means running cable to every wet spot in the house; the Wi-Fi sensor needs recharging, and basements are exactly where Wi-Fi is weakest.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -5560,7 +5572,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 1 – PoE wired IP camera with ONVIF/RTSP. It dominates the highest-weighted criteria: connection reliability (dedicated cable, no Wi-Fi drop-outs), local recording with open standards (streams directly to the local server/NVR without any vendor cloud), zero Wi-Fi bandwidth impact, and power over the same cable from a UPS-backed PoE switch. Its only weakness is installation complexity (cable runs), accepted as a one-time cost. Analog HD coax is cheap and reliable but limited in resolution and integration; Wi-Fi mains cameras congest the home network; Wi-Fi battery cameras need frequent charging, record only on motion events and usually lock recordings into a cloud subscription.</t>
+          <t>Option 1, PoE wired IP cameras with ONVIF/RTSP, with a total of 4.30. The criteria I weighted highest were connection reliability and local, open-standard recording, and PoE wins both without much discussion: one cable carries power and video, the NVR on the CCU records without any vendor cloud, and the cameras keep running from the UPS-backed PoE switch during a power cut. The price for that is installation effort (cable runs), which I scored a 2 and accept as a one-off cost. The analog HD coax option surprised me by coming second: it is cheap and reliable, but it needs a separate DVR and integrates poorly. Wi-Fi mains cameras congest the home network; Wi-Fi battery cameras need charging every few weeks, record only on motion and usually lock the recordings into a subscription.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -6980,7 +6992,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 1 – Zigbee smart lock. It scores best on the three top-weighted criteria taken together: native protocol fit with the Zigbee hub (no extra radio), fully offline operation through local automations, and solid security with Zigbee 3.0 AES-128 link keys plus tamper and low-battery reporting, with battery life of many months. The Z-Wave lock offers S2 security but requires an additional Z-Wave controller and costs more. The Wi-Fi lock drains its battery within weeks and typically depends on the vendor cloud to operate.</t>
+          <t>Option 1, a Zigbee smart lock. For a lock I weighted security, offline operation and protocol fit highest. The Zigbee lock works entirely through the CCU's local automations (auto-lock on Armed Away) with no internet involved, reports tamper and low battery, and uses the same AES-128 link keys as the sensors. The Z-Wave lock is a close second with its S2 security class, but it would be the only Z-Wave device in the house and would need its own controller. The Wi-Fi lock I would not put on my own front door: the battery lasts weeks and most models stop working when the vendor cloud is down.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -8400,7 +8412,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 1 – Zigbee smart bulb / switch. It fits the Zigbee hub natively, is controlled locally without internet, responds instantly to alarm scenes (flash all lights on intrusion) and – because mains-powered Zigbee devices act as mesh routers – every light strengthens the coverage of the battery sensor network. Wi-Fi smart plugs are cheap but on/off only, add Wi-Fi load and often depend on the vendor cloud. Z-Wave in-wall switches need in-wall wiring and a second radio, and do not extend the Zigbee mesh.</t>
+          <t>Option 1, Zigbee bulbs and switches, by a wide margin (4.85). Beyond the obvious points (native hub fit, local control, instant response to alarm scenes) there is a side benefit that decided it: mains-powered Zigbee devices are mesh routers, so every bulb I add makes the battery sensors' network stronger. Wi-Fi plugs are cheap and fine for non-security loads, but they are on/off only and usually cloud-dependent. Z-Wave in-wall switches need an electrician and a second radio, and do nothing for the Zigbee mesh.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -9805,7 +9817,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 2 – Wired 12 V siren on a CCU relay output, as the primary outdoor sounder. It scores highest on the two heaviest criteria – loudness (110+ dB outdoor siren with strobe) and reliability during a power or Wi-Fi outage – because it is driven directly by the battery-backed CCU through an end-of-line supervised, tamper-protected loop. The Zigbee indoor siren scored almost as high thanks to its easy installation and native hub fit, so the system uses BOTH: a Zigbee indoor siren for in-home alerting plus a wired 12 V outdoor siren + strobe for deterrence and neighbour notification. The Wi-Fi siren is rejected because it falls silent exactly when the network fails.</t>
+          <t>This is the one matrix where the winner on paper is not the whole answer. The wired 12 V siren scores highest (4.20) because loudness and reliability during a power or network outage are the heaviest criteria, and a siren hanging off the battery-backed CCU through a supervised, tamper-protected loop is as reliable as it gets. The Zigbee indoor siren is only a tenth behind thanks to easy installation and hub fit. So the design uses both: a Zigbee siren indoors (quick to fit, loud enough at 95 dB) and a wired 12 V siren with strobe outdoors for deterrence and so the neighbours notice. The Wi-Fi siren was never a serious candidate; it goes quiet exactly when the network fails, which is when you need it.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -11253,7 +11265,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Selected: Option 3 – Hybrid: local-first server with a thin cloud relay. All alarm logic, sensor processing, automations and video recording run on the on-premises server, so alarm response latency and operation during an internet outage are as good as the local-only design and far better than cloud-only, where the home is unprotected the moment the ISP link drops. The cloud component is deliberately minimal: an outbound-only, TLS-encrypted relay for remote app access and push notifications, plus an encrypted off-site backup of configuration and event logs. This keeps personal data and video inside the home (privacy 4/5 versus 1/5 for a vendor cloud), avoids inbound port forwarding (a smaller attack surface than a home-exposed local server), and keeps recurring cost low because no video is stored in the cloud. Local-only was a close second but fails on remote access convenience – a user-configured VPN with no push notifications is not acceptable for a consumer security product – and has no off-site backup if the server is stolen or destroyed. Cloud-only wins on upfront cost, maintenance and scalability but is rejected on the highest-weighted criteria: outage reliability, privacy, recurring 5-year cost and attack surface.</t>
+          <t>Option 3, the hybrid local-first server with a thin cloud relay (3.95), ahead of local-only (3.70) and cloud-only (2.45). I spent most of my trade-off time on this matrix because every other decision depends on it. Everything that matters for safety (sensor processing, alarm logic, automations, recording) runs on the mini PC in the house, so alarm latency and behaviour during an internet outage are identical to the local-only design and nothing like cloud-only, where the house is unprotected the moment the ISP link drops. The cloud part is deliberately small: an outbound TLS relay so the app and push notifications work from anywhere without opening ports on the router, plus an encrypted off-site copy of configuration and event logs. That keeps video and personal data at home (I scored privacy 4 against 1 for a vendor cloud), keeps the attack surface smaller than a home-exposed server, and keeps running costs low because no video goes to the cloud. Local-only was genuinely close and I went back and forth on it; what sank it was remote access: asking a family to configure a VPN and giving up push notifications is not realistic for a consumer product, and a stolen server takes the only copy of the logs with it. Cloud-only wins on upfront cost, maintenance and scalability, but loses on the criteria I weighted most: outage behaviour, privacy, 5-year cost and attack surface.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>

</xml_diff>

<commit_message>
Tidy README and wording in the SysRS and decision matrices
</commit_message>
<xml_diff>
--- a/04-Decision-Matrix/SHSS_Decision_Matrices.xlsx
+++ b/04-Decision-Matrix/SHSS_Decision_Matrices.xlsx
@@ -748,7 +748,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>The scores are my own judgement from data sheets, product reviews and, for a few of the devices, hands-on use. I filled in the weights first and the scores afterwards so that the weighting could not be tuned towards a favourite option. Where two options were close I say so in the final-decision text instead of pretending the numbers settle it.</t>
+          <t>The scores are my own judgement based on typical published specifications for devices in each class; they are estimates, not measurements. Where two options are close the final-decision text says so rather than pretending the numbers settle it.</t>
         </is>
       </c>
     </row>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Option 1, a Zigbee smart lock. For a lock I weighted security, offline operation and protocol fit highest. The Zigbee lock works entirely through the CCU's local automations (auto-lock on Armed Away) with no internet involved, reports tamper and low battery, and uses the same AES-128 link keys as the sensors. The Z-Wave lock is a close second with its S2 security class, but it would be the only Z-Wave device in the house and would need its own controller. The Wi-Fi lock I would not put on my own front door: the battery lasts weeks and most models stop working when the vendor cloud is down.</t>
+          <t>Option 1, a Zigbee smart lock. For a lock I weighted security, offline operation and protocol fit highest. The Zigbee lock works entirely through the CCU's local automations (auto-lock on Armed Away) with no internet involved, reports tamper and low battery, and uses the same AES-128 link keys as the sensors. The Z-Wave lock is a close second with its S2 security class, but it would be the only Z-Wave device in the house and would need its own controller. The Wi-Fi lock is the weakest option: the battery lasts weeks and most models stop working when the vendor cloud is down.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -11265,7 +11265,7 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Option 3, the hybrid local-first server with a thin cloud relay (3.95), ahead of local-only (3.70) and cloud-only (2.45). I spent most of my trade-off time on this matrix because every other decision depends on it. Everything that matters for safety (sensor processing, alarm logic, automations, recording) runs on the mini PC in the house, so alarm latency and behaviour during an internet outage are identical to the local-only design and nothing like cloud-only, where the house is unprotected the moment the ISP link drops. The cloud part is deliberately small: an outbound TLS relay so the app and push notifications work from anywhere without opening ports on the router, plus an encrypted off-site copy of configuration and event logs. That keeps video and personal data at home (I scored privacy 4 against 1 for a vendor cloud), keeps the attack surface smaller than a home-exposed server, and keeps running costs low because no video goes to the cloud. Local-only was genuinely close and I went back and forth on it; what sank it was remote access: asking a family to configure a VPN and giving up push notifications is not realistic for a consumer product, and a stolen server takes the only copy of the logs with it. Cloud-only wins on upfront cost, maintenance and scalability, but loses on the criteria I weighted most: outage behaviour, privacy, 5-year cost and attack surface.</t>
+          <t>Option 3, the hybrid local-first server with a thin cloud relay (3.95), ahead of local-only (3.70) and cloud-only (2.45). This is the matrix every other decision depends on, which is why it has the most criteria. Everything that matters for safety (sensor processing, alarm logic, automations, recording) runs on the mini PC in the house, so alarm latency and behaviour during an internet outage are identical to the local-only design and nothing like cloud-only, where the house is unprotected the moment the ISP link drops. The cloud part is deliberately small: an outbound TLS relay so the app and push notifications work from anywhere without opening ports on the router, plus an encrypted off-site copy of configuration and event logs. That keeps video and personal data at home (I scored privacy 4 against 1 for a vendor cloud), keeps the attack surface smaller than a home-exposed server, and keeps running costs low because no video goes to the cloud. Local-only was genuinely close; what decided it was remote access: asking a family to configure a VPN and giving up push notifications is not realistic for a consumer product, and a stolen server takes the only copy of the logs with it. Cloud-only wins on upfront cost, maintenance and scalability, but loses on the criteria I weighted most: outage behaviour, privacy, 5-year cost and attack surface.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>

</xml_diff>